<commit_message>
Bug cálculo tiempo reacción arreglado
</commit_message>
<xml_diff>
--- a/datosPreguntasReaccion.xlsx
+++ b/datosPreguntasReaccion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hlocal\C_TFG\Datos\Mision Colombia-20260209T150018Z-3-001\jsonToCsv_TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7240B81-0643-4D8C-869C-2662ABA2A2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E16787F-D44C-4C5A-8FAF-66D2D88B6647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -745,7 +745,7 @@
     <t>14:17:38.331</t>
   </si>
   <si>
-    <t>14:17:44.930</t>
+    <t>14:18:35.700</t>
   </si>
   <si>
     <t>14:18:36.653</t>
@@ -4882,7 +4882,7 @@
     <t>14:47:48.528</t>
   </si>
   <si>
-    <t>14:50:51.851</t>
+    <t>15:11:56.541</t>
   </si>
   <si>
     <t>15:12:03.577</t>
@@ -9172,7 +9172,7 @@
     <t>14:20:59.161</t>
   </si>
   <si>
-    <t>14:21:00.727</t>
+    <t>14:21:51.864</t>
   </si>
   <si>
     <t>14:21:54.550</t>
@@ -11737,7 +11737,7 @@
     <t>15:14:30.933</t>
   </si>
   <si>
-    <t>15:14:37.531</t>
+    <t>15:16:35.553</t>
   </si>
   <si>
     <t>15:16:42.772</t>
@@ -16152,9 +16152,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -16173,7 +16171,50 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -16184,6 +16225,24 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E031E6AD-F931-4416-B97D-BB7FF0E2200E}" name="Tabla2" displayName="Tabla2" ref="A1:I3114" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:I3114" xr:uid="{E031E6AD-F931-4416-B97D-BB7FF0E2200E}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{018E221B-E8FB-43C3-8E4A-693ABB827F6A}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{50D9167F-0837-4DB1-9D45-DBA3CCD423B8}" name="Sesion"/>
+    <tableColumn id="3" xr3:uid="{8C5A0731-3B06-4D9A-B225-C2E9022CDAF4}" name="Nivel"/>
+    <tableColumn id="4" xr3:uid="{0FBD29EB-131C-42A4-94A9-03A90F1BA658}" name="Intento"/>
+    <tableColumn id="5" xr3:uid="{E328A79A-F0FE-4164-B8B8-2E2107A55A3D}" name="Tipo"/>
+    <tableColumn id="6" xr3:uid="{8B7655B7-F1A7-425C-96E7-AFE270452CA5}" name="Tiempo inicio"/>
+    <tableColumn id="7" xr3:uid="{C242E1AA-28EB-4C51-B8E8-D2F3565198FF}" name="Tiempo respuesta"/>
+    <tableColumn id="8" xr3:uid="{7E7EBA95-6578-4890-BD70-C7029610AFD7}" name="Tiempo reaccion(s)"/>
+    <tableColumn id="9" xr3:uid="{09C62543-0516-4A94-AE89-81C7EB48A73A}" name="Respuesta"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16473,6 +16532,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I3114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="17.77734375" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -20027,7 +20093,7 @@
         <v>242</v>
       </c>
       <c r="H128">
-        <v>51.722999999999999</v>
+        <v>0.95299999999999996</v>
       </c>
       <c r="I128" t="s">
         <v>12</v>
@@ -42088,7 +42154,7 @@
         <v>1621</v>
       </c>
       <c r="H936">
-        <v>1271.7260000000001</v>
+        <v>7.0359999999999996</v>
       </c>
       <c r="I936" t="s">
         <v>12</v>
@@ -64846,7 +64912,7 @@
         <v>3051</v>
       </c>
       <c r="H1764">
-        <v>53.823</v>
+        <v>2.6859999999999999</v>
       </c>
       <c r="I1764" t="s">
         <v>12</v>
@@ -78587,7 +78653,7 @@
         <v>3906</v>
       </c>
       <c r="H2264">
-        <v>125.241</v>
+        <v>7.2190000000000003</v>
       </c>
       <c r="I2264" t="s">
         <v>12</v>
@@ -101847,5 +101913,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>